<commit_message>
feat: add unit encyclopedia and battle content updates
</commit_message>
<xml_diff>
--- a/docs/excel/unit_data.xlsx
+++ b/docs/excel/unit_data.xlsx
@@ -194,12 +194,12 @@
     <t>—</t>
   </si>
   <si>
-    <t>造成追击后，下回合开始时获得+1金币（每场战斗仅生效1次）</t>
-  </si>
-  <si>
     <t>造成追击后，下回合开始时获得+2金币（每场战斗仅生效1次）</t>
   </si>
   <si>
+    <t>造成追击后，下回合开始时获得+4金币（每场战斗仅生效1次）</t>
+  </si>
+  <si>
     <t>经济/远程辅助；先机速度按职业而非星级</t>
   </si>
   <si>
@@ -272,10 +272,10 @@
     <t>骑士</t>
   </si>
   <si>
-    <t>回合开始时，如果场上至少有5支甘地部队，本部队临时数量+（5*回合数）。</t>
-  </si>
-  <si>
-    <t>回合开始时，如果场上至少有5支甘地部队，本部队临时数量+（10*回合数）。</t>
+    <t>回合结束时，如果场上至少有5支甘地部队，本部队临时数量+（5*回合数）。</t>
+  </si>
+  <si>
+    <t>回合结束时，如果场上至少有5支甘地部队，本部队临时数量+（10*回合数）。</t>
   </si>
   <si>
     <t>开战后，瞬间冲到最近的敌人，造成1次暴击伤害和1轮的眩晕</t>
@@ -314,10 +314,10 @@
     <t>每入场5支甘地部队，随机获得2支甘地部队</t>
   </si>
   <si>
-    <t>开战后，随机给友方2支部队增加一个护盾，护盾可以完全抵挡最多1次的伤害</t>
-  </si>
-  <si>
-    <t>开战后，随机给友方4支部队增加一个护盾，护盾可以完全抵挡最多1次的伤害</t>
+    <t>开战后，给队伍最前面存在友方部队的1排的所有友方部队增加一个护盾，护盾可以完全抵挡最多1次的伤害</t>
+  </si>
+  <si>
+    <t>开战后，给队伍最前面存在友方部队的2排的所有友方部队增加一个护盾，护盾可以完全抵挡最多1次的伤害</t>
   </si>
   <si>
     <t>护盾辅助</t>
@@ -338,10 +338,10 @@
     <t>武学大师</t>
   </si>
   <si>
-    <t>每获得1支甘地部队，本部队+2数量（购买、发现、随机获得均计入）。</t>
-  </si>
-  <si>
-    <t>每获得1支甘地部队，本部队+4数量（购买、发现、随机获得均计入）。</t>
+    <t>每获得1支甘地部队，本部队+2数量（购买、发现、随机获得均计入）。回合结束时，同排战士获得+2数量。</t>
+  </si>
+  <si>
+    <t>每获得1支甘地部队，本部队+4数量（购买、发现、随机获得均计入）。回合结束时，同排战士获得+4数量。</t>
   </si>
   <si>
     <t>每次攻击都会造成周围1距离内的范围伤害</t>
@@ -368,10 +368,10 @@
     <t>卫戍协兵</t>
   </si>
   <si>
-    <t>任意友军获得1次补员时，全军获得+1数量。</t>
-  </si>
-  <si>
-    <t>任意友军获得1次补员时，全军获得+2数量。</t>
+    <t>回合结束时，当前所在的排以及身后的所有排的单位均获得+1数量，同时触发1次所有战士的回合结束效果</t>
+  </si>
+  <si>
+    <t>回合结束时，当前所在的排以及身后的所有排的单位均获得+2数量，同时触发2次所有战士的回合结束效果</t>
   </si>
   <si>
     <t>我方任意部队产生1次暴击，本部队临时数量+10。</t>
@@ -398,10 +398,10 @@
     <t>皇家剑士</t>
   </si>
   <si>
-    <t>回合结束时，全体战士+1数量。</t>
-  </si>
-  <si>
-    <t>回合结束时，全体战士+2数量。</t>
+    <t>回合结束时，全体战士+1数量。与自己同一排的所有单位也可视为战士。</t>
+  </si>
+  <si>
+    <t>回合结束时，全体战士+2数量。与自己同一排的所有单位也可视为战士。</t>
   </si>
   <si>
     <t>高阶重装战士</t>
@@ -979,10 +979,10 @@
     <t>蘑菇夸库</t>
   </si>
   <si>
-    <t>回合结束时，临时获得左右两侧部队中当前数量较高一方的数量。</t>
-  </si>
-  <si>
-    <t>回合结束时，临时获得本排和前一排部队中当前数量较高一方的数量。</t>
+    <t>回合结束时，临时获得左右两侧部队中当前数量较高一方的数量的一半。</t>
+  </si>
+  <si>
+    <t>回合结束时，临时获得本排和前一排部队中当前数量较高一方的数量的一半。</t>
   </si>
   <si>
     <t>雪狮</t>
@@ -2561,7 +2561,7 @@
         <v>3</v>
       </c>
       <c r="O3" s="13">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P3" s="13">
         <v>0</v>

</xml_diff>